<commit_message>
pulizia di label, spazi, maiuscole e separatori (T-85, D-023)
Spazi finali in 4 label e 3 descrizioni, U+00A0 in 5 ancoraggi,
adjacentto, close_reading, separatori di Alternative_Toponym.
Nessun valore semantico cambia; 16.029 / 17.187 triple, SHACL conforme.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/NarrativePlaces.xlsx
+++ b/data/source/xlsx/NarrativePlaces.xlsx
@@ -1663,7 +1663,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Il complesso, progettato dall'architetto Innocenzo Costantini, si estendeva su tutta l'area di Piazza Pepe, sulla quale si affaccia anche il famoso Teatro Ambra Jovinelli.[5] La struttura, sorta nel pieno periodo fascista (1929), era inoltre disposta nel cortile dove troneggiava l'Acquedotto Giulio (Aqua Iulia).</t>
+          <t>Il complesso, progettato dall'architetto Innocenzo Costantini, si estendeva su tutta l'area di Piazza Pepe, sulla quale si affaccia anche il famoso Teatro Ambra Jovinelli.[5] La struttura, sorta nel pieno periodo fascista (1929), era inoltre disposta nel cortile dove troneggiava l'Acquedotto Giulio (Aqua Iulia).</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Espressione evocativa usata come sineddoche spaziale dell’origine sociale e culturale del personaggio; non luogo diegetico </t>
+          <t>Espressione evocativa usata come sineddoche spaziale dell’origine sociale e culturale del personaggio; non luogo diegetico</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2638,7 +2638,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>antro;botteguccia; bottega;</t>
+          <t>antro; botteguccia; bottega</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -3382,7 +3382,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Luogo non precisato simile a un orto o una vigna, di fronte al laboratorio della Zamira, al lato opposto della via Appia </t>
+          <t>Luogo non precisato simile a un orto o una vigna, di fronte al laboratorio della Zamira, al lato opposto della via Appia</t>
         </is>
       </c>
       <c r="I115" t="n">
@@ -3478,7 +3478,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Palazzo </t>
+          <t>Palazzo</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3505,7 +3505,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>palazzo dell'oro;palazzo de li pescicani; ben nota architettura; casermone color pidocchio; sto palazzo; camere al duecentodiciannove; il duecentodiciannove</t>
+          <t>palazzo dell'oro; palazzo de li pescicani; ben nota architettura; casermone color pidocchio; sto palazzo; camere al duecentodiciannove; il duecentodiciannove</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3829,7 +3829,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Piazza Colonna </t>
+          <t>Piazza Colonna</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -6772,7 +6772,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Via dei Greci </t>
+          <t>Via dei Greci</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -7222,7 +7222,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t xml:space="preserve">Via Lanza </t>
+          <t>Via Lanza</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">

</xml_diff>

<commit_message>
Casal Bruciato: luogo trasformato con ancoraggio relazionale (T-15, D-025)
Nessuna coordinata reale: ancore Marino, Albano, Pavona, Santa Palomba,
con la lettura di Manzotti (2010, pp. 268–270) come nota critica.
Eliminata gaz_casal_bruciato (quartiere romano, referente errato);
il casello diventa parte di Casal Bruciato. ABox 16.029 -> 16.044,
full 17.187 -> 17.202, SHACL conforme. Chiude DC-18.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/NarrativePlaces.xlsx
+++ b/data/source/xlsx/NarrativePlaces.xlsx
@@ -1364,7 +1364,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>imported</t>
+          <t>transformed</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Quartiere di Roma</t>
+          <t>Luogo trasformato, senza coordinate proprie: località dell'agro romano circoscritta da Marino e dall'Appia verso Albano (nord/nord-est), da Pavona (ovest) e da Santa Palomba (sud). Non è il quartiere romano omonimo.</t>
         </is>
       </c>
     </row>
@@ -1392,6 +1392,11 @@
       <c r="D39" t="inlineStr">
         <is>
           <t>transformed</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>casal_bruciato</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">

</xml_diff>

<commit_message>
permutazione Invented <-> Imagined in TBox e dati (T-04, D-026)
Definizioni SKOS scambiate secondo Reuschel, Piatti e Hurni (2013),
skos:notation 1-4, scopeNote, commento di hasRealityStatus,
owl:differentFrom completi; scambio atomico dei valori nei TSV.
Invented 15, Imagined 5. TBox 588 -> 600, full 17.202 -> 17.214,
SHACL conforme. Glifi non toccati (T-65).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/NarrativePlaces.xlsx
+++ b/data/source/xlsx/NarrativePlaces.xlsx
@@ -984,7 +984,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>invented</t>
+          <t>imagined</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>invented</t>
+          <t>imagined</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -2648,7 +2648,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>invented</t>
+          <t>imagined</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -3372,7 +3372,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -3777,7 +3777,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>invented</t>
+          <t>imagined</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -5751,7 +5751,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>invented</t>
+          <t>imagined</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
@@ -6204,7 +6204,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">

</xml_diff>

<commit_message>
Edicola ai Due Santi: luogo importato con ancoraggio derivato (T-03, D-027)
Nuova gaz_edicola_due_santi: posizione di Due Santi con uno scarto
dichiarato di ~40 m, fonte Manzotti 2010, p. 246. Tolto Is_Part_Of.
ABox 16.044 -> 16.055, full 17.214 -> 17.225, SHACL conforme.
Chiude DC-03.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/NarrativePlaces.xlsx
+++ b/data/source/xlsx/NarrativePlaces.xlsx
@@ -2118,12 +2118,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>invented</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>orto_vigna_due_santi</t>
+          <t>imported</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -2133,7 +2128,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Edicola immaginata al di sopra del muro di cinta della vigna/orto sul lato opposto della via Appia rispetto al laboratorio della Zamira</t>
+          <t>Tabernacolo a due pioventi che interrompe il muriccio dell'orto o vigna di fronte al laboratorio della Zamira, sul lato opposto della via Appia (QP 216, 219). Luogo importato: Manzotti (2010, p. 246) ne trova traccia nella piantina dei Castelli del Touring.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Casal Bruciato: casale reale, Imported, con posizioni TCI e IGM (D-033, rivede D-025; D-034)
Nuova gaz_casale_abbruciato nella posizione TCI adottata (Manzotti
2010, Tav. VI); IGM alternativa in nota (Tav. VII). Ancore per passo
(Castel di Leva, Divino Amore, Falcognana, Roma–Velletri, Ardeatina,
Santa Palomba); tolti Marino e Albano; Pavona come inferenza di Manzotti.
Riferimento aggiunto per QP 241. Casello ancorato alla Roma–Velletri.
Adapter: ancora principale = referente del luogo (D-034).
ABox 16.057 -> 16.093, full 17.227 -> 17.263, statuti 260/30/14/5,
SHACL conforme. Chiude DC-18.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/NarrativePlaces.xlsx
+++ b/data/source/xlsx/NarrativePlaces.xlsx
@@ -1362,9 +1362,14 @@
           <t>Casal Bruciato</t>
         </is>
       </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Casale Abbrusciato</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>transformed</t>
+          <t>imported</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1374,7 +1379,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Luogo trasformato, senza coordinate proprie: località dell'agro romano circoscritta da Marino e dall'Appia verso Albano (nord/nord-est), da Pavona (ovest) e da Santa Palomba (sud). Non è il quartiere romano omonimo.</t>
+          <t>Casale reale dell'Agro romano a sud di Roma (Casal(e) Bruciato / Abbruciato / Abbrusciato: Nibby, Dintorni di Roma, p. 569), fra le ferrovie Roma–Velletri e Roma–Napoli. Non è il quartiere omonimo del Tiburtino. Forme attestate: «Casal Bruciato» (QP 212, 237, 240, 241, 262, 274, 298), «Casale Abbrusciato» (QP 297).</t>
         </is>
       </c>
     </row>
@@ -1392,11 +1397,6 @@
       <c r="D39" t="inlineStr">
         <is>
           <t>transformed</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>casal_bruciato</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">

</xml_diff>

<commit_message>
astensione dall'ancoraggio a tre valori, distinta dal dato mancante (T-35, D-048)
LocalizationStatusScheme (analisi non condotta, sospensione motivata,
coordinata non applicabile); default: 5 Imagined -> non applicabile,
12 luoghi senza ancoraggio -> analisi non condotta. Shape 10, IQ14.
TBox 971 -> 1.013, ABox 25.755 -> 25.772, SHACL conforme.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/NarrativePlaces.xlsx
+++ b/data/source/xlsx/NarrativePlaces.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I310"/>
+  <dimension ref="A1:K310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,16 @@
           <t>Fuzziness_Level</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Localization_Status</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Localization_Reason</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1350,6 +1360,11 @@
           <t>Casa immaginata nella zona dei Due Santi</t>
         </is>
       </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>non applicabile</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1529,6 +1544,11 @@
           <t>Castello d'immaginazione, deformazione linguistica di Castel Porziano</t>
         </is>
       </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>non applicabile</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1796,6 +1816,11 @@
           <t>località</t>
         </is>
       </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>analisi non condotta</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1900,6 +1925,11 @@
           <t>monumento</t>
         </is>
       </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>analisi non condotta</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2273,6 +2303,11 @@
           <t>fontanella</t>
         </is>
       </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>analisi non condotta</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2317,6 +2352,11 @@
           <t>complesso sportivo</t>
         </is>
       </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>analisi non condotta</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2433,6 +2473,11 @@
           <t>palazzo storico</t>
         </is>
       </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>analisi non condotta</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2806,6 +2851,11 @@
           <t>via</t>
         </is>
       </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>analisi non condotta</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3151,6 +3201,11 @@
           <t>Monte inventato, collocato nella zona dei Colli Albani/marino</t>
         </is>
       </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>non applicabile</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3935,6 +3990,11 @@
           <t>piazza</t>
         </is>
       </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>analisi non condotta</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4067,6 +4127,11 @@
           <t>piazza</t>
         </is>
       </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>analisi non condotta</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -4496,6 +4561,11 @@
           <t>quartiere</t>
         </is>
       </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>analisi non condotta</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -4611,6 +4681,11 @@
           <t>località</t>
         </is>
       </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>analisi non condotta</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -4820,6 +4895,11 @@
           <t>località</t>
         </is>
       </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>non applicabile</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -4899,6 +4979,11 @@
           <t>catacombe</t>
         </is>
       </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>analisi non condotta</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -5767,6 +5852,11 @@
       <c r="I214" t="n">
         <v>3</v>
       </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>non applicabile</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -5983,6 +6073,11 @@
       <c r="F223" t="inlineStr">
         <is>
           <t>sito archeologico</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>analisi non condotta</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ancoraggio relazionale; regola di geometria; elenco fuori carta (T-47, D-057)
RelationalAnchoring con termini e tipo (near, between). Casal Bruciato:
posizione solo dal casale (TCI), luoghi intorno come termini near. Robine
Vecchie: una interpretazione «tra» Frattocchie e Due Santi, senza posizione,
sospensione motivata; doppione 00473 eliminato (960 -> 959). L'adapter mette
i luoghi senza posizione adottata in offMap (pannello T-62). Shape 17.
TBox 1.158 -> 1.187, ABox 27.136 -> 27.144, feature 301 -> 300.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/NarrativePlaces.xlsx
+++ b/data/source/xlsx/NarrativePlaces.xlsx
@@ -4801,6 +4801,16 @@
           <t>Robine Vecchie è un microtoponimo gaddiano non identificato, forse deformazione di un nome locale o denominazione fantastica applicata al paesaggio reale di Frattocchie–Due Santi.</t>
         </is>
       </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>sospensione motivata</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>Solo ancoraggio relazionale: il passo colloca le Robine Vecchie fra Frattocchie e Due Santi (QP 169), senza una posizione. Toponimo «non registrato nelle carte topografiche» (Terzoli 2015, p. 491).</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">

</xml_diff>

<commit_message>
forma attestata sull'occorrenza, soprannomi sul luogo (T-48, D-059)
chora:attestedForm (178 occorrenze, sottostringhe esatte degli estratti),
chora:nickname (palazzo de li pescicani, er palazzo dell'oro); varianti li
Du Santi, Castel Savelli, Castel Porcino come altLabel; una forma per
letterale. Shape 18.
TBox 1.217 -> 1.230, ABox 27.148 -> 27.336, SHACL conforme.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/NarrativePlaces.xlsx
+++ b/data/source/xlsx/NarrativePlaces.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K310"/>
+  <dimension ref="A1:L310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,11 @@
           <t>Localization_Reason</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Nickname</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1526,7 +1531,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>castel porcino</t>
+          <t>Castel Porcino</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1561,6 +1566,11 @@
           <t>Castel Savello</t>
         </is>
       </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Castel Savelli</t>
+        </is>
+      </c>
       <c r="D45" t="inlineStr">
         <is>
           <t>imported</t>
@@ -2109,6 +2119,11 @@
           <t>Due Santi</t>
         </is>
       </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>li Du Santi</t>
+        </is>
+      </c>
       <c r="D67" t="inlineStr">
         <is>
           <t>imported</t>
@@ -3560,7 +3575,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>palazzo dell'oro; palazzo de li pescicani; ben nota architettura; casermone color pidocchio; sto palazzo; camere al duecentodiciannove; il duecentodiciannove</t>
+          <t>ben nota architettura;casermone color pidocchio;sto palazzo;camere al duecentodiciannove;il duecentodiciannove</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3576,6 +3591,11 @@
       <c r="G120" t="inlineStr">
         <is>
           <t>Luogo che identifica il palazzo in via Merulana 219</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>palazzo de li pescicani;er palazzo dell'oro</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
difetti della TBox: non applicabile, interpretazione, agenti, mapping (D-062)
NotApplicable non deriva più dallo statuto: tolti i 5 valori dei luoghi
Imagined, da assegnare da Lorenzo. Definizione di SpatialInterpretation
corretta. Agenti prov:Person con classe Scholar/Annotator; shape 20.
Sezione documentation in mapping.yaml per i fogli letti dal codice.
TBox 1.307 -> 1.320, ABox 27.854 -> 27.863, SHACL conforme.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/NarrativePlaces.xlsx
+++ b/data/source/xlsx/NarrativePlaces.xlsx
@@ -1365,11 +1365,6 @@
           <t>Casa immaginata nella zona dei Due Santi</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>non applicabile</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1549,11 +1544,6 @@
           <t>Castello d'immaginazione, deformazione linguistica di Castel Porziano</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>non applicabile</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3216,11 +3206,6 @@
           <t>Monte inventato, collocato nella zona dei Colli Albani/marino</t>
         </is>
       </c>
-      <c r="J107" t="inlineStr">
-        <is>
-          <t>non applicabile</t>
-        </is>
-      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4925,11 +4910,6 @@
           <t>località</t>
         </is>
       </c>
-      <c r="J175" t="inlineStr">
-        <is>
-          <t>non applicabile</t>
-        </is>
-      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -5881,11 +5861,6 @@
       </c>
       <c r="I214" t="n">
         <v>3</v>
-      </c>
-      <c r="J214" t="inlineStr">
-        <is>
-          <t>non applicabile</t>
-        </is>
       </c>
     </row>
     <row r="215">

</xml_diff>

<commit_message>
nessun luogo annotato fuori dall'interfaccia, corregge D-057 (blocco F, D-084)
Termini relazionali del gazetteer come ancore quando mancano ancore
dirette (Robine Vecchie torna in carta); offMap e sospensione tolti;
controlli permanenti: IQ21 e shape 23 (Violation), audit bloccante sulla
presenza di ogni luogo annotato nel GeoJSON. Feature 300 -> 301.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/NarrativePlaces.xlsx
+++ b/data/source/xlsx/NarrativePlaces.xlsx
@@ -4806,16 +4806,6 @@
           <t>Robine Vecchie è un microtoponimo gaddiano non identificato, forse deformazione di un nome locale o denominazione fantastica applicata al paesaggio reale di Frattocchie–Due Santi.</t>
         </is>
       </c>
-      <c r="J171" t="inlineStr">
-        <is>
-          <t>sospensione motivata</t>
-        </is>
-      </c>
-      <c r="K171" t="inlineStr">
-        <is>
-          <t>Solo ancoraggio relazionale: il passo colloca le Robine Vecchie fra Frattocchie e Due Santi (QPa 169), senza una posizione. Toponimo «non registrato nelle carte topografiche» (Terzoli 2015, p. 491).</t>
-        </is>
-      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">

</xml_diff>

<commit_message>
Fase 3b, B1: cinque luoghi Imagined diventano Invented (D-090)
Nuove letture S-<luogo>-2 adottate che rivedono S-<luogo> (prov:wasRevisionOf);
le letture Imagined restano nel grafo, non adottate.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/NarrativePlaces.xlsx
+++ b/data/source/xlsx/NarrativePlaces.xlsx
@@ -1352,7 +1352,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3193,7 +3193,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -4892,7 +4892,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -5836,7 +5836,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>imagined</t>
+          <t>invented</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">

</xml_diff>

<commit_message>
Fase 3c, B1: cantina della Zamira, sacello responsale, camera di sicurezza della questura (D-091)
Otto occorrenze con estratti verificati da LS sul volume a stampa, undici
interpretazioni, due letture di statuto, tre membri di P-0001, due semi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/NarrativePlaces.xlsx
+++ b/data/source/xlsx/NarrativePlaces.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L311"/>
+  <dimension ref="A1:L314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8131,6 +8131,107 @@
         </is>
       </c>
     </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>cantina_zamira</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Cantina della Zamira</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>sala di tintoria; salotto o sala di consultazione; antro</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>invented</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>casuccia_zamira</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>interno</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>Cantina o sala seminterrata sotto il laboratorio della Zamira, sala delle consultazioni (QPa 165, 166). Luogo entrato con la soglia di censimento (D-091).</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>sacello_responsale</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Sacello responsale</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>invented</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>casuccia_zamira</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>interno</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>Sacello o ricettacolo responsale della Zamira, a cui la sala di consultazione dà adito per un uscio con catenaccio (QPa 165). Luogo entrato con la soglia di censimento (D-091).</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>camera_sicurezza_questura</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Camera di sicurezza della questura</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>imported</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>santo_stefano_del_cacco_celio_santo_stefano</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>camera</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>Camera di sicurezza della questura di Santo Stefano del Cacco, dove Ines attende l'alba (QPa 176). Luogo entrato con la soglia di censimento (D-091).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>